<commit_message>
feat: add MPS API sync for work order customer and shipping date
</commit_message>
<xml_diff>
--- a/Newdata/成品報工.XLSX
+++ b/Newdata/成品報工.XLSX
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="184">
-  <si>
-    <t>100003438</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1667" uniqueCount="232">
+  <si>
+    <t>100003496</t>
   </si>
   <si>
     <t>0</t>
@@ -40,7 +40,7 @@
     <t>PP01</t>
   </si>
   <si>
-    <t>1377318</t>
+    <t>1403784</t>
   </si>
   <si>
     <t>REL</t>
@@ -58,10 +58,10 @@
     <t>主軸馬達安裝</t>
   </si>
   <si>
-    <t>1377329</t>
-  </si>
-  <si>
-    <t>100003449</t>
+    <t>1403794</t>
+  </si>
+  <si>
+    <t>100003508</t>
   </si>
   <si>
     <t>6</t>
@@ -76,13 +76,88 @@
     <t>馬達動平衡校正</t>
   </si>
   <si>
-    <t>1379722</t>
-  </si>
-  <si>
-    <t>100003451</t>
-  </si>
-  <si>
-    <t>0394</t>
+    <t>1414691</t>
+  </si>
+  <si>
+    <t>100003534</t>
+  </si>
+  <si>
+    <t>1429824</t>
+  </si>
+  <si>
+    <t>100003535</t>
+  </si>
+  <si>
+    <t>1430037</t>
+  </si>
+  <si>
+    <t>100003536</t>
+  </si>
+  <si>
+    <t>1430250</t>
+  </si>
+  <si>
+    <t>100003537</t>
+  </si>
+  <si>
+    <t>1430463</t>
+  </si>
+  <si>
+    <t>100003543</t>
+  </si>
+  <si>
+    <t>0200</t>
+  </si>
+  <si>
+    <t>1432135</t>
+  </si>
+  <si>
+    <t>100003544</t>
+  </si>
+  <si>
+    <t>1432354</t>
+  </si>
+  <si>
+    <t>100003545</t>
+  </si>
+  <si>
+    <t>1432573</t>
+  </si>
+  <si>
+    <t>100003546</t>
+  </si>
+  <si>
+    <t>1432792</t>
+  </si>
+  <si>
+    <t>100003547</t>
+  </si>
+  <si>
+    <t>1433011</t>
+  </si>
+  <si>
+    <t>100003548</t>
+  </si>
+  <si>
+    <t>1433230</t>
+  </si>
+  <si>
+    <t>100003553</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>0190</t>
+  </si>
+  <si>
+    <t>1540003</t>
+  </si>
+  <si>
+    <t>旋臂座介面座清潔</t>
+  </si>
+  <si>
+    <t>1436359</t>
   </si>
   <si>
     <t>1540009</t>
@@ -91,10 +166,10 @@
     <t>旋臂組清潔除漆</t>
   </si>
   <si>
-    <t>1380249</t>
-  </si>
-  <si>
-    <t>0396</t>
+    <t>1436360</t>
+  </si>
+  <si>
+    <t>0210</t>
   </si>
   <si>
     <t>1540010</t>
@@ -103,10 +178,10 @@
     <t>旋臂零組件組裝</t>
   </si>
   <si>
-    <t>1380250</t>
-  </si>
-  <si>
-    <t>0398</t>
+    <t>1436361</t>
+  </si>
+  <si>
+    <t>0220</t>
   </si>
   <si>
     <t>1540008</t>
@@ -115,352 +190,421 @@
     <t>油電系統組裝</t>
   </si>
   <si>
-    <t>1380251</t>
-  </si>
-  <si>
-    <t>100003470</t>
-  </si>
-  <si>
-    <t>1387952</t>
-  </si>
-  <si>
-    <t>100003471</t>
-  </si>
-  <si>
-    <t>1388157</t>
-  </si>
-  <si>
-    <t>100003473</t>
+    <t>1436362</t>
+  </si>
+  <si>
+    <t>100003559</t>
+  </si>
+  <si>
+    <t>1439653</t>
+  </si>
+  <si>
+    <t>1439654</t>
+  </si>
+  <si>
+    <t>1439655</t>
+  </si>
+  <si>
+    <t>0230</t>
+  </si>
+  <si>
+    <t>1439656</t>
+  </si>
+  <si>
+    <t>100003560</t>
+  </si>
+  <si>
+    <t>0270</t>
+  </si>
+  <si>
+    <t>3050001</t>
+  </si>
+  <si>
+    <t>刀庫安裝</t>
+  </si>
+  <si>
+    <t>1439868</t>
+  </si>
+  <si>
+    <t>0850</t>
+  </si>
+  <si>
+    <t>3050007</t>
+  </si>
+  <si>
+    <t>刀庫調整</t>
+  </si>
+  <si>
+    <t>1439911</t>
+  </si>
+  <si>
+    <t>0860</t>
+  </si>
+  <si>
+    <t>3050002</t>
+  </si>
+  <si>
+    <t>刀庫合刀作業</t>
+  </si>
+  <si>
+    <t>1439912</t>
+  </si>
+  <si>
+    <t>0170</t>
+  </si>
+  <si>
+    <t>1439974</t>
+  </si>
+  <si>
+    <t>100003562</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1560007</t>
+  </si>
+  <si>
+    <t>頭倉底座組清潔</t>
+  </si>
+  <si>
+    <t>1440639</t>
+  </si>
+  <si>
+    <t>1560008</t>
+  </si>
+  <si>
+    <t>頭倉定位水平校正</t>
+  </si>
+  <si>
+    <t>1440640</t>
+  </si>
+  <si>
+    <t>0240</t>
+  </si>
+  <si>
+    <t>1560009</t>
+  </si>
+  <si>
+    <t>零組件清潔裝配</t>
+  </si>
+  <si>
+    <t>1440641</t>
+  </si>
+  <si>
+    <t>0250</t>
+  </si>
+  <si>
+    <t>1560010</t>
+  </si>
+  <si>
+    <t>馬達座精度磨配</t>
+  </si>
+  <si>
+    <t>1440642</t>
+  </si>
+  <si>
+    <t>0260</t>
+  </si>
+  <si>
+    <t>1560011</t>
+  </si>
+  <si>
+    <t>軸承座精度磨配</t>
+  </si>
+  <si>
+    <t>1440643</t>
+  </si>
+  <si>
+    <t>1560012</t>
+  </si>
+  <si>
+    <t>進給座精度磨配</t>
+  </si>
+  <si>
+    <t>1440644</t>
+  </si>
+  <si>
+    <t>0280</t>
+  </si>
+  <si>
+    <t>1560013</t>
+  </si>
+  <si>
+    <t>頭倉打PIN作業</t>
+  </si>
+  <si>
+    <t>1440645</t>
+  </si>
+  <si>
+    <t>0290</t>
+  </si>
+  <si>
+    <t>1560014</t>
+  </si>
+  <si>
+    <t>角度頭倉機構裝配</t>
+  </si>
+  <si>
+    <t>1440646</t>
+  </si>
+  <si>
+    <t>0300</t>
+  </si>
+  <si>
+    <t>1560015</t>
+  </si>
+  <si>
+    <t>鈑金系統裝配</t>
+  </si>
+  <si>
+    <t>1440647</t>
+  </si>
+  <si>
+    <t>1560016</t>
+  </si>
+  <si>
+    <t>伸縮護蓋裝配</t>
+  </si>
+  <si>
+    <t>1440648</t>
+  </si>
+  <si>
+    <t>0320</t>
+  </si>
+  <si>
+    <t>1560017</t>
+  </si>
+  <si>
+    <t>周邊裝配及防銹</t>
+  </si>
+  <si>
+    <t>1440649</t>
+  </si>
+  <si>
+    <t>100003563</t>
+  </si>
+  <si>
+    <t>0670</t>
+  </si>
+  <si>
+    <t>1442779</t>
+  </si>
+  <si>
+    <t>100003564</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>1442594</t>
+  </si>
+  <si>
+    <t>100003568</t>
+  </si>
+  <si>
+    <t>0281</t>
+  </si>
+  <si>
+    <t>1443844</t>
+  </si>
+  <si>
+    <t>100003572</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>0190</t>
-  </si>
-  <si>
-    <t>1390304</t>
-  </si>
-  <si>
-    <t>100003474</t>
-  </si>
-  <si>
-    <t>0170</t>
-  </si>
-  <si>
-    <t>1390405</t>
-  </si>
-  <si>
-    <t>100003475</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>1390493</t>
-  </si>
-  <si>
-    <t>100003481</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>0210</t>
-  </si>
-  <si>
-    <t>1394060</t>
-  </si>
-  <si>
-    <t>0220</t>
-  </si>
-  <si>
-    <t>1394061</t>
-  </si>
-  <si>
-    <t>0230</t>
-  </si>
-  <si>
-    <t>1394062</t>
-  </si>
-  <si>
-    <t>100003482</t>
-  </si>
-  <si>
-    <t>0200</t>
-  </si>
-  <si>
-    <t>1540003</t>
-  </si>
-  <si>
-    <t>旋臂座介面座清潔</t>
-  </si>
-  <si>
-    <t>1394413</t>
-  </si>
-  <si>
-    <t>1394414</t>
-  </si>
-  <si>
-    <t>1394415</t>
-  </si>
-  <si>
-    <t>1394416</t>
-  </si>
-  <si>
-    <t>100003483</t>
-  </si>
-  <si>
-    <t>1394767</t>
-  </si>
-  <si>
-    <t>1394768</t>
-  </si>
-  <si>
-    <t>1394769</t>
-  </si>
-  <si>
-    <t>1394770</t>
-  </si>
-  <si>
-    <t>100003496</t>
-  </si>
-  <si>
-    <t>1403784</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>0340</t>
-  </si>
-  <si>
-    <t>1403788</t>
-  </si>
-  <si>
-    <t>1403794</t>
-  </si>
-  <si>
-    <t>100003504</t>
-  </si>
-  <si>
-    <t>1407414</t>
-  </si>
-  <si>
-    <t>1407415</t>
-  </si>
-  <si>
-    <t>1407416</t>
-  </si>
-  <si>
-    <t>1407417</t>
-  </si>
-  <si>
-    <t>100003507</t>
-  </si>
-  <si>
-    <t>1411454</t>
-  </si>
-  <si>
-    <t>100003508</t>
-  </si>
-  <si>
-    <t>1414691</t>
-  </si>
-  <si>
-    <t>100003509</t>
-  </si>
-  <si>
-    <t>1414896</t>
-  </si>
-  <si>
-    <t>100003510</t>
-  </si>
-  <si>
-    <t>1415194</t>
-  </si>
-  <si>
-    <t>1415195</t>
-  </si>
-  <si>
-    <t>1415196</t>
-  </si>
-  <si>
-    <t>1415197</t>
-  </si>
-  <si>
-    <t>100003515</t>
-  </si>
-  <si>
-    <t>1416109</t>
-  </si>
-  <si>
-    <t>100003521</t>
-  </si>
-  <si>
-    <t>1422599</t>
-  </si>
-  <si>
-    <t>100003522</t>
-  </si>
-  <si>
-    <t>1422700</t>
-  </si>
-  <si>
-    <t>100003523</t>
-  </si>
-  <si>
-    <t>1426157</t>
-  </si>
-  <si>
-    <t>100003524</t>
-  </si>
-  <si>
-    <t>1426254</t>
-  </si>
-  <si>
-    <t>100003525</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>1426821</t>
-  </si>
-  <si>
-    <t>100003526</t>
-  </si>
-  <si>
-    <t>1427454</t>
-  </si>
-  <si>
-    <t>100003527</t>
-  </si>
-  <si>
-    <t>1428430</t>
-  </si>
-  <si>
-    <t>100003534</t>
-  </si>
-  <si>
-    <t>1429824</t>
-  </si>
-  <si>
-    <t>100003535</t>
-  </si>
-  <si>
-    <t>1430037</t>
-  </si>
-  <si>
-    <t>100003536</t>
-  </si>
-  <si>
-    <t>1430250</t>
-  </si>
-  <si>
-    <t>100003537</t>
-  </si>
-  <si>
-    <t>1430463</t>
-  </si>
-  <si>
-    <t>100003538</t>
-  </si>
-  <si>
-    <t>1431484</t>
-  </si>
-  <si>
-    <t>100003539</t>
-  </si>
-  <si>
-    <t>1431584</t>
-  </si>
-  <si>
-    <t>100003540</t>
-  </si>
-  <si>
-    <t>1431684</t>
-  </si>
-  <si>
-    <t>100003541</t>
-  </si>
-  <si>
-    <t>1431777</t>
-  </si>
-  <si>
-    <t>100003542</t>
-  </si>
-  <si>
-    <t>1431916</t>
-  </si>
-  <si>
-    <t>100003543</t>
-  </si>
-  <si>
-    <t>1432135</t>
-  </si>
-  <si>
-    <t>100003544</t>
-  </si>
-  <si>
-    <t>1432354</t>
-  </si>
-  <si>
-    <t>100003545</t>
-  </si>
-  <si>
-    <t>1432573</t>
-  </si>
-  <si>
-    <t>100003546</t>
-  </si>
-  <si>
-    <t>1432792</t>
-  </si>
-  <si>
-    <t>100003547</t>
-  </si>
-  <si>
-    <t>1433011</t>
-  </si>
-  <si>
-    <t>100003548</t>
-  </si>
-  <si>
-    <t>1433230</t>
-  </si>
-  <si>
-    <t>100003553</t>
-  </si>
-  <si>
-    <t>1436359</t>
-  </si>
-  <si>
-    <t>1436360</t>
-  </si>
-  <si>
-    <t>1436361</t>
-  </si>
-  <si>
-    <t>1436362</t>
-  </si>
-  <si>
-    <t>100003554</t>
-  </si>
-  <si>
-    <t>1436473</t>
-  </si>
-  <si>
-    <t>100003555</t>
-  </si>
-  <si>
-    <t>1436573</t>
-  </si>
-  <si>
-    <t>100003556</t>
-  </si>
-  <si>
-    <t>1437074</t>
+    <t>1444654</t>
+  </si>
+  <si>
+    <t>100003573</t>
+  </si>
+  <si>
+    <t>1444858</t>
+  </si>
+  <si>
+    <t>100003574</t>
+  </si>
+  <si>
+    <t>1445062</t>
+  </si>
+  <si>
+    <t>100003578</t>
+  </si>
+  <si>
+    <t>1445878</t>
+  </si>
+  <si>
+    <t>100003579</t>
+  </si>
+  <si>
+    <t>1446082</t>
+  </si>
+  <si>
+    <t>100003580</t>
+  </si>
+  <si>
+    <t>1446286</t>
+  </si>
+  <si>
+    <t>100003585</t>
+  </si>
+  <si>
+    <t>1449017</t>
+  </si>
+  <si>
+    <t>100003587</t>
+  </si>
+  <si>
+    <t>1453060</t>
+  </si>
+  <si>
+    <t>100003590</t>
+  </si>
+  <si>
+    <t>1453659</t>
+  </si>
+  <si>
+    <t>100003593</t>
+  </si>
+  <si>
+    <t>1453959</t>
+  </si>
+  <si>
+    <t>100003595</t>
+  </si>
+  <si>
+    <t>1457817</t>
+  </si>
+  <si>
+    <t>100003596</t>
+  </si>
+  <si>
+    <t>1457917</t>
+  </si>
+  <si>
+    <t>100003597</t>
+  </si>
+  <si>
+    <t>1458017</t>
+  </si>
+  <si>
+    <t>100003598</t>
+  </si>
+  <si>
+    <t>1458117</t>
+  </si>
+  <si>
+    <t>100003599</t>
+  </si>
+  <si>
+    <t>1458217</t>
+  </si>
+  <si>
+    <t>100003600</t>
+  </si>
+  <si>
+    <t>1458348</t>
+  </si>
+  <si>
+    <t>100003601</t>
+  </si>
+  <si>
+    <t>1458428</t>
+  </si>
+  <si>
+    <t>100003602</t>
+  </si>
+  <si>
+    <t>1458741</t>
+  </si>
+  <si>
+    <t>100003603</t>
+  </si>
+  <si>
+    <t>1458945</t>
+  </si>
+  <si>
+    <t>100003604</t>
+  </si>
+  <si>
+    <t>1459035</t>
+  </si>
+  <si>
+    <t>100003606</t>
+  </si>
+  <si>
+    <t>1460616</t>
+  </si>
+  <si>
+    <t>100003607</t>
+  </si>
+  <si>
+    <t>1461381</t>
+  </si>
+  <si>
+    <t>100003608</t>
+  </si>
+  <si>
+    <t>1461469</t>
+  </si>
+  <si>
+    <t>100003609</t>
+  </si>
+  <si>
+    <t>1461569</t>
+  </si>
+  <si>
+    <t>100003610</t>
+  </si>
+  <si>
+    <t>1461670</t>
+  </si>
+  <si>
+    <t>100003612</t>
+  </si>
+  <si>
+    <t>1463036</t>
+  </si>
+  <si>
+    <t>100003614</t>
+  </si>
+  <si>
+    <t>1463491</t>
+  </si>
+  <si>
+    <t>100003616</t>
+  </si>
+  <si>
+    <t>1465072</t>
+  </si>
+  <si>
+    <t>100003617</t>
+  </si>
+  <si>
+    <t>1466583</t>
+  </si>
+  <si>
+    <t>100003618</t>
+  </si>
+  <si>
+    <t>1466683</t>
+  </si>
+  <si>
+    <t>100003619</t>
+  </si>
+  <si>
+    <t>1466783</t>
+  </si>
+  <si>
+    <t>100003621</t>
+  </si>
+  <si>
+    <t>1469385</t>
   </si>
   <si>
     <t>訂單</t>
@@ -676,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AH67"/>
+  <dimension ref="A1:AH72"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="11" customWidth="1"/>
@@ -717,106 +861,106 @@
   <sheetData>
     <row r="1" spans="1:34">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>151</v>
+        <v>199</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>152</v>
+        <v>200</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>203</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>156</v>
+        <v>204</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>157</v>
+        <v>205</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>158</v>
+        <v>206</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>159</v>
+        <v>207</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>161</v>
+        <v>209</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>162</v>
+        <v>210</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>163</v>
+        <v>211</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>164</v>
+        <v>212</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>165</v>
+        <v>213</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>166</v>
+        <v>214</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>167</v>
+        <v>215</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>168</v>
+        <v>216</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>169</v>
+        <v>217</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>170</v>
+        <v>218</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>171</v>
+        <v>219</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>175</v>
+        <v>223</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>179</v>
+        <v>227</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>181</v>
+        <v>229</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:34">
@@ -1127,7 +1271,7 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
         <v>3</v>
@@ -1136,10 +1280,10 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>
@@ -1148,13 +1292,13 @@
         <v>7</v>
       </c>
       <c r="J5" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K5" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="L5" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="M5" t="s">
         <v>8</v>
@@ -1175,7 +1319,7 @@
         <v>0.000</v>
       </c>
       <c r="S5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
@@ -1221,13 +1365,13 @@
     </row>
     <row r="6" spans="1:34">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
         <v>3</v>
@@ -1236,10 +1380,10 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
@@ -1248,13 +1392,13 @@
         <v>7</v>
       </c>
       <c r="J6" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K6" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L6" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M6" t="s">
         <v>8</v>
@@ -1275,7 +1419,7 @@
         <v>0.000</v>
       </c>
       <c r="S6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
@@ -1321,13 +1465,13 @@
     </row>
     <row r="7" spans="1:34">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
         <v>3</v>
@@ -1336,10 +1480,10 @@
         <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2">
         <v>1</v>
@@ -1348,13 +1492,13 @@
         <v>7</v>
       </c>
       <c r="J7" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K7" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L7" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M7" t="s">
         <v>8</v>
@@ -1375,7 +1519,7 @@
         <v>0.000</v>
       </c>
       <c r="S7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="T7" s="5"/>
       <c r="U7" s="5"/>
@@ -1421,7 +1565,7 @@
     </row>
     <row r="8" spans="1:34">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
@@ -1475,7 +1619,7 @@
         <v>0.000</v>
       </c>
       <c r="S8" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="T8" s="5"/>
       <c r="U8" s="5"/>
@@ -1521,13 +1665,13 @@
     </row>
     <row r="9" spans="1:34">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
         <v>3</v>
@@ -1575,7 +1719,7 @@
         <v>0.000</v>
       </c>
       <c r="S9" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
@@ -1621,13 +1765,13 @@
     </row>
     <row r="10" spans="1:34">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
         <v>3</v>
@@ -1675,7 +1819,7 @@
         <v>0.000</v>
       </c>
       <c r="S10" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
@@ -1721,13 +1865,13 @@
     </row>
     <row r="11" spans="1:34">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
         <v>3</v>
@@ -1775,7 +1919,7 @@
         <v>0.000</v>
       </c>
       <c r="S11" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
@@ -1821,13 +1965,13 @@
     </row>
     <row r="12" spans="1:34">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -1875,7 +2019,7 @@
         <v>0.000</v>
       </c>
       <c r="S12" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="T12" s="5"/>
       <c r="U12" s="5"/>
@@ -1921,13 +2065,13 @@
     </row>
     <row r="13" spans="1:34">
       <c r="A13" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
         <v>3</v>
@@ -1936,10 +2080,10 @@
         <v>4</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H13" s="2">
         <v>1</v>
@@ -1948,13 +2092,13 @@
         <v>7</v>
       </c>
       <c r="J13" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K13" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="L13" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="M13" t="s">
         <v>8</v>
@@ -1975,7 +2119,7 @@
         <v>0.000</v>
       </c>
       <c r="S13" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
@@ -2021,13 +2165,13 @@
     </row>
     <row r="14" spans="1:34">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
         <v>3</v>
@@ -2036,10 +2180,10 @@
         <v>4</v>
       </c>
       <c r="F14" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H14" s="2">
         <v>1</v>
@@ -2048,13 +2192,13 @@
         <v>7</v>
       </c>
       <c r="J14" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K14" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L14" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M14" t="s">
         <v>8</v>
@@ -2075,7 +2219,7 @@
         <v>0.000</v>
       </c>
       <c r="S14" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="T14" s="5"/>
       <c r="U14" s="5"/>
@@ -2121,13 +2265,13 @@
     </row>
     <row r="15" spans="1:34">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
         <v>3</v>
@@ -2136,10 +2280,10 @@
         <v>4</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H15" s="2">
         <v>1</v>
@@ -2148,13 +2292,13 @@
         <v>7</v>
       </c>
       <c r="J15" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="K15" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="L15" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="M15" t="s">
         <v>8</v>
@@ -2175,7 +2319,7 @@
         <v>0.000</v>
       </c>
       <c r="S15" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="T15" s="5"/>
       <c r="U15" s="5"/>
@@ -2221,13 +2365,13 @@
     </row>
     <row r="16" spans="1:34">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
         <v>3</v>
@@ -2236,10 +2380,10 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H16" s="2">
         <v>1</v>
@@ -2248,13 +2392,13 @@
         <v>7</v>
       </c>
       <c r="J16" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K16" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="L16" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M16" t="s">
         <v>8</v>
@@ -2275,7 +2419,7 @@
         <v>0.000</v>
       </c>
       <c r="S16" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
@@ -2321,13 +2465,13 @@
     </row>
     <row r="17" spans="1:34">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
         <v>3</v>
@@ -2336,10 +2480,10 @@
         <v>4</v>
       </c>
       <c r="F17" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="G17" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="H17" s="2">
         <v>1</v>
@@ -2348,13 +2492,13 @@
         <v>7</v>
       </c>
       <c r="J17" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="K17" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="L17" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="M17" t="s">
         <v>8</v>
@@ -2375,7 +2519,7 @@
         <v>0.000</v>
       </c>
       <c r="S17" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="T17" s="5"/>
       <c r="U17" s="5"/>
@@ -2421,13 +2565,13 @@
     </row>
     <row r="18" spans="1:34">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
         <v>3</v>
@@ -2436,10 +2580,10 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="G18" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="H18" s="2">
         <v>1</v>
@@ -2475,7 +2619,7 @@
         <v>0.000</v>
       </c>
       <c r="S18" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="T18" s="5"/>
       <c r="U18" s="5"/>
@@ -2521,13 +2665,13 @@
     </row>
     <row r="19" spans="1:34">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D19" t="s">
         <v>3</v>
@@ -2536,10 +2680,10 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G19" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="H19" s="2">
         <v>1</v>
@@ -2548,13 +2692,13 @@
         <v>7</v>
       </c>
       <c r="J19" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="K19" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="L19" s="3">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="M19" t="s">
         <v>8</v>
@@ -2575,7 +2719,7 @@
         <v>0.000</v>
       </c>
       <c r="S19" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="T19" s="5"/>
       <c r="U19" s="5"/>
@@ -2621,13 +2765,13 @@
     </row>
     <row r="20" spans="1:34">
       <c r="A20" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
         <v>3</v>
@@ -2636,10 +2780,10 @@
         <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G20" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H20" s="2">
         <v>1</v>
@@ -2648,13 +2792,13 @@
         <v>7</v>
       </c>
       <c r="J20" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K20" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="L20" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M20" t="s">
         <v>8</v>
@@ -2675,7 +2819,7 @@
         <v>0.000</v>
       </c>
       <c r="S20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="T20" s="5"/>
       <c r="U20" s="5"/>
@@ -2721,13 +2865,13 @@
     </row>
     <row r="21" spans="1:34">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D21" t="s">
         <v>3</v>
@@ -2736,10 +2880,10 @@
         <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="G21" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="H21" s="2">
         <v>1</v>
@@ -2748,13 +2892,13 @@
         <v>7</v>
       </c>
       <c r="J21" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="K21" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="L21" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="M21" t="s">
         <v>8</v>
@@ -2775,7 +2919,7 @@
         <v>0.000</v>
       </c>
       <c r="S21" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
@@ -2821,13 +2965,13 @@
     </row>
     <row r="22" spans="1:34">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
         <v>3</v>
@@ -2836,10 +2980,10 @@
         <v>4</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="H22" s="2">
         <v>1</v>
@@ -2875,7 +3019,7 @@
         <v>0.000</v>
       </c>
       <c r="S22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
@@ -2921,13 +3065,13 @@
     </row>
     <row r="23" spans="1:34">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="D23" t="s">
         <v>3</v>
@@ -2936,10 +3080,10 @@
         <v>4</v>
       </c>
       <c r="F23" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="G23" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="H23" s="2">
         <v>1</v>
@@ -2975,7 +3119,7 @@
         <v>0.000</v>
       </c>
       <c r="S23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="T23" s="5"/>
       <c r="U23" s="5"/>
@@ -3021,13 +3165,13 @@
     </row>
     <row r="24" spans="1:34">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="D24" t="s">
         <v>3</v>
@@ -3036,10 +3180,10 @@
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="G24" t="s">
-        <v>6</v>
+        <v>73</v>
       </c>
       <c r="H24" s="2">
         <v>1</v>
@@ -3075,7 +3219,7 @@
         <v>0.000</v>
       </c>
       <c r="S24" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="T24" s="5"/>
       <c r="U24" s="5"/>
@@ -3121,13 +3265,13 @@
     </row>
     <row r="25" spans="1:34">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D25" t="s">
         <v>3</v>
@@ -3136,10 +3280,10 @@
         <v>4</v>
       </c>
       <c r="F25" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="G25" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="H25" s="2">
         <v>1</v>
@@ -3148,13 +3292,13 @@
         <v>7</v>
       </c>
       <c r="J25" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="K25" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="L25" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="M25" t="s">
         <v>8</v>
@@ -3175,7 +3319,7 @@
         <v>0.000</v>
       </c>
       <c r="S25" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="T25" s="5"/>
       <c r="U25" s="5"/>
@@ -3221,13 +3365,13 @@
     </row>
     <row r="26" spans="1:34">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B26" t="s">
         <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="D26" t="s">
         <v>3</v>
@@ -3236,10 +3380,10 @@
         <v>4</v>
       </c>
       <c r="F26" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G26" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H26" s="2">
         <v>1</v>
@@ -3248,13 +3392,13 @@
         <v>7</v>
       </c>
       <c r="J26" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K26" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L26" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M26" t="s">
         <v>8</v>
@@ -3275,7 +3419,7 @@
         <v>0.000</v>
       </c>
       <c r="S26" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="T26" s="5"/>
       <c r="U26" s="5"/>
@@ -3321,13 +3465,13 @@
     </row>
     <row r="27" spans="1:34">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D27" t="s">
         <v>3</v>
@@ -3336,10 +3480,10 @@
         <v>4</v>
       </c>
       <c r="F27" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="G27" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="H27" s="2">
         <v>1</v>
@@ -3348,13 +3492,13 @@
         <v>7</v>
       </c>
       <c r="J27" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="K27" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="L27" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M27" t="s">
         <v>8</v>
@@ -3375,7 +3519,7 @@
         <v>0.000</v>
       </c>
       <c r="S27" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="T27" s="5"/>
       <c r="U27" s="5"/>
@@ -3421,13 +3565,13 @@
     </row>
     <row r="28" spans="1:34">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D28" t="s">
         <v>3</v>
@@ -3436,10 +3580,10 @@
         <v>4</v>
       </c>
       <c r="F28" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
       <c r="G28" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="H28" s="2">
         <v>1</v>
@@ -3448,13 +3592,13 @@
         <v>7</v>
       </c>
       <c r="J28" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="K28" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="L28" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="M28" t="s">
         <v>8</v>
@@ -3475,7 +3619,7 @@
         <v>0.000</v>
       </c>
       <c r="S28" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="T28" s="5"/>
       <c r="U28" s="5"/>
@@ -3521,13 +3665,13 @@
     </row>
     <row r="29" spans="1:34">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B29" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="D29" t="s">
         <v>3</v>
@@ -3536,10 +3680,10 @@
         <v>4</v>
       </c>
       <c r="F29" t="s">
-        <v>28</v>
+        <v>90</v>
       </c>
       <c r="G29" t="s">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="H29" s="2">
         <v>1</v>
@@ -3575,7 +3719,7 @@
         <v>0.000</v>
       </c>
       <c r="S29" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
@@ -3621,13 +3765,13 @@
     </row>
     <row r="30" spans="1:34">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B30" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>93</v>
       </c>
       <c r="D30" t="s">
         <v>3</v>
@@ -3636,10 +3780,10 @@
         <v>4</v>
       </c>
       <c r="F30" t="s">
-        <v>32</v>
+        <v>94</v>
       </c>
       <c r="G30" t="s">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="H30" s="2">
         <v>1</v>
@@ -3675,7 +3819,7 @@
         <v>0.000</v>
       </c>
       <c r="S30" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="T30" s="5"/>
       <c r="U30" s="5"/>
@@ -3724,10 +3868,10 @@
         <v>81</v>
       </c>
       <c r="B31" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C31" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
         <v>3</v>
@@ -3736,10 +3880,10 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="G31" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="H31" s="2">
         <v>1</v>
@@ -3748,13 +3892,13 @@
         <v>7</v>
       </c>
       <c r="J31" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="K31" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="L31" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="M31" t="s">
         <v>8</v>
@@ -3775,7 +3919,7 @@
         <v>0.000</v>
       </c>
       <c r="S31" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
@@ -3821,13 +3965,13 @@
     </row>
     <row r="32" spans="1:34">
       <c r="A32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B32" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
         <v>3</v>
@@ -3836,10 +3980,10 @@
         <v>4</v>
       </c>
       <c r="F32" t="s">
-        <v>19</v>
+        <v>101</v>
       </c>
       <c r="G32" t="s">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="H32" s="2">
         <v>1</v>
@@ -3848,13 +3992,13 @@
         <v>7</v>
       </c>
       <c r="J32" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="K32" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="L32" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="M32" t="s">
         <v>8</v>
@@ -3875,7 +4019,7 @@
         <v>0.000</v>
       </c>
       <c r="S32" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="T32" s="5"/>
       <c r="U32" s="5"/>
@@ -3921,13 +4065,13 @@
     </row>
     <row r="33" spans="1:34">
       <c r="A33" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B33" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
+        <v>104</v>
       </c>
       <c r="D33" t="s">
         <v>3</v>
@@ -3936,10 +4080,10 @@
         <v>4</v>
       </c>
       <c r="F33" t="s">
-        <v>19</v>
+        <v>105</v>
       </c>
       <c r="G33" t="s">
-        <v>20</v>
+        <v>106</v>
       </c>
       <c r="H33" s="2">
         <v>1</v>
@@ -3948,13 +4092,13 @@
         <v>7</v>
       </c>
       <c r="J33" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="K33" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="L33" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="M33" t="s">
         <v>8</v>
@@ -3975,7 +4119,7 @@
         <v>0.000</v>
       </c>
       <c r="S33" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="T33" s="5"/>
       <c r="U33" s="5"/>
@@ -4021,13 +4165,13 @@
     </row>
     <row r="34" spans="1:34">
       <c r="A34" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B34" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C34" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
       <c r="D34" t="s">
         <v>3</v>
@@ -4036,10 +4180,10 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
       <c r="G34" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="H34" s="2">
         <v>1</v>
@@ -4048,13 +4192,13 @@
         <v>7</v>
       </c>
       <c r="J34" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="K34" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="L34" s="3">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M34" t="s">
         <v>8</v>
@@ -4075,7 +4219,7 @@
         <v>0.000</v>
       </c>
       <c r="S34" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="T34" s="5"/>
       <c r="U34" s="5"/>
@@ -4121,13 +4265,13 @@
     </row>
     <row r="35" spans="1:34">
       <c r="A35" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C35" t="s">
-        <v>51</v>
+        <v>112</v>
       </c>
       <c r="D35" t="s">
         <v>3</v>
@@ -4136,10 +4280,10 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>24</v>
+        <v>113</v>
       </c>
       <c r="G35" t="s">
-        <v>25</v>
+        <v>114</v>
       </c>
       <c r="H35" s="2">
         <v>1</v>
@@ -4148,13 +4292,13 @@
         <v>7</v>
       </c>
       <c r="J35" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="K35" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="L35" s="3">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="M35" t="s">
         <v>8</v>
@@ -4175,7 +4319,7 @@
         <v>0.000</v>
       </c>
       <c r="S35" t="s">
-        <v>89</v>
+        <v>115</v>
       </c>
       <c r="T35" s="5"/>
       <c r="U35" s="5"/>
@@ -4221,13 +4365,13 @@
     </row>
     <row r="36" spans="1:34">
       <c r="A36" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="D36" t="s">
         <v>3</v>
@@ -4236,10 +4380,10 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="G36" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="H36" s="2">
         <v>1</v>
@@ -4275,7 +4419,7 @@
         <v>0.000</v>
       </c>
       <c r="S36" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="T36" s="5"/>
       <c r="U36" s="5"/>
@@ -4321,13 +4465,13 @@
     </row>
     <row r="37" spans="1:34">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="C37" t="s">
-        <v>55</v>
+        <v>119</v>
       </c>
       <c r="D37" t="s">
         <v>3</v>
@@ -4336,10 +4480,10 @@
         <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="G37" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
       <c r="H37" s="2">
         <v>1</v>
@@ -4348,13 +4492,13 @@
         <v>7</v>
       </c>
       <c r="J37" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="K37" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="L37" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M37" t="s">
         <v>8</v>
@@ -4375,7 +4519,7 @@
         <v>0.000</v>
       </c>
       <c r="S37" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="T37" s="5"/>
       <c r="U37" s="5"/>
@@ -4421,13 +4565,13 @@
     </row>
     <row r="38" spans="1:34">
       <c r="A38" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="B38" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
       <c r="D38" t="s">
         <v>3</v>
@@ -4436,10 +4580,10 @@
         <v>4</v>
       </c>
       <c r="F38" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="G38" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="H38" s="2">
         <v>1</v>
@@ -4448,13 +4592,13 @@
         <v>7</v>
       </c>
       <c r="J38" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="K38" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="L38" s="3">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="M38" t="s">
         <v>8</v>
@@ -4475,7 +4619,7 @@
         <v>0.000</v>
       </c>
       <c r="S38" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="T38" s="5"/>
       <c r="U38" s="5"/>
@@ -4521,13 +4665,13 @@
     </row>
     <row r="39" spans="1:34">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>127</v>
       </c>
       <c r="C39" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="D39" t="s">
         <v>3</v>
@@ -4575,7 +4719,7 @@
         <v>0.000</v>
       </c>
       <c r="S39" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="T39" s="5"/>
       <c r="U39" s="5"/>
@@ -4621,13 +4765,13 @@
     </row>
     <row r="40" spans="1:34">
       <c r="A40" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>44</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
         <v>3</v>
@@ -4675,7 +4819,7 @@
         <v>0.000</v>
       </c>
       <c r="S40" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="T40" s="5"/>
       <c r="U40" s="5"/>
@@ -4721,13 +4865,13 @@
     </row>
     <row r="41" spans="1:34">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D41" t="s">
         <v>3</v>
@@ -4775,7 +4919,7 @@
         <v>0.000</v>
       </c>
       <c r="S41" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="T41" s="5"/>
       <c r="U41" s="5"/>
@@ -4821,13 +4965,13 @@
     </row>
     <row r="42" spans="1:34">
       <c r="A42" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C42" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D42" t="s">
         <v>3</v>
@@ -4875,7 +5019,7 @@
         <v>0.000</v>
       </c>
       <c r="S42" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="T42" s="5"/>
       <c r="U42" s="5"/>
@@ -4921,13 +5065,13 @@
     </row>
     <row r="43" spans="1:34">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
       <c r="B43" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="C43" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D43" t="s">
         <v>3</v>
@@ -4975,7 +5119,7 @@
         <v>0.000</v>
       </c>
       <c r="S43" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
       <c r="T43" s="5"/>
       <c r="U43" s="5"/>
@@ -5021,13 +5165,13 @@
     </row>
     <row r="44" spans="1:34">
       <c r="A44" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="C44" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D44" t="s">
         <v>3</v>
@@ -5075,7 +5219,7 @@
         <v>0.000</v>
       </c>
       <c r="S44" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="T44" s="5"/>
       <c r="U44" s="5"/>
@@ -5121,13 +5265,13 @@
     </row>
     <row r="45" spans="1:34">
       <c r="A45" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C45" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D45" t="s">
         <v>3</v>
@@ -5175,7 +5319,7 @@
         <v>0.000</v>
       </c>
       <c r="S45" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="T45" s="5"/>
       <c r="U45" s="5"/>
@@ -5221,13 +5365,13 @@
     </row>
     <row r="46" spans="1:34">
       <c r="A46" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="B46" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C46" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D46" t="s">
         <v>3</v>
@@ -5275,7 +5419,7 @@
         <v>0.000</v>
       </c>
       <c r="S46" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
@@ -5321,7 +5465,7 @@
     </row>
     <row r="47" spans="1:34">
       <c r="A47" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="B47" t="s">
         <v>17</v>
@@ -5375,7 +5519,7 @@
         <v>0.000</v>
       </c>
       <c r="S47" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="T47" s="5"/>
       <c r="U47" s="5"/>
@@ -5421,13 +5565,13 @@
     </row>
     <row r="48" spans="1:34">
       <c r="A48" t="s">
-        <v>113</v>
+        <v>148</v>
       </c>
       <c r="B48" t="s">
-        <v>17</v>
+        <v>127</v>
       </c>
       <c r="C48" t="s">
-        <v>18</v>
+        <v>79</v>
       </c>
       <c r="D48" t="s">
         <v>3</v>
@@ -5475,7 +5619,7 @@
         <v>0.000</v>
       </c>
       <c r="S48" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>
@@ -5521,13 +5665,13 @@
     </row>
     <row r="49" spans="1:34">
       <c r="A49" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="B49" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C49" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="D49" t="s">
         <v>3</v>
@@ -5575,7 +5719,7 @@
         <v>0.000</v>
       </c>
       <c r="S49" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="T49" s="5"/>
       <c r="U49" s="5"/>
@@ -5621,13 +5765,13 @@
     </row>
     <row r="50" spans="1:34">
       <c r="A50" t="s">
-        <v>117</v>
+        <v>152</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C50" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D50" t="s">
         <v>3</v>
@@ -5675,7 +5819,7 @@
         <v>0.000</v>
       </c>
       <c r="S50" t="s">
-        <v>118</v>
+        <v>153</v>
       </c>
       <c r="T50" s="5"/>
       <c r="U50" s="5"/>
@@ -5721,13 +5865,13 @@
     </row>
     <row r="51" spans="1:34">
       <c r="A51" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="B51" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C51" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D51" t="s">
         <v>3</v>
@@ -5775,7 +5919,7 @@
         <v>0.000</v>
       </c>
       <c r="S51" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="T51" s="5"/>
       <c r="U51" s="5"/>
@@ -5821,13 +5965,13 @@
     </row>
     <row r="52" spans="1:34">
       <c r="A52" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="B52" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C52" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D52" t="s">
         <v>3</v>
@@ -5875,7 +6019,7 @@
         <v>0.000</v>
       </c>
       <c r="S52" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="T52" s="5"/>
       <c r="U52" s="5"/>
@@ -5921,13 +6065,13 @@
     </row>
     <row r="53" spans="1:34">
       <c r="A53" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="B53" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C53" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D53" t="s">
         <v>3</v>
@@ -5975,7 +6119,7 @@
         <v>0.000</v>
       </c>
       <c r="S53" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="T53" s="5"/>
       <c r="U53" s="5"/>
@@ -6021,13 +6165,13 @@
     </row>
     <row r="54" spans="1:34">
       <c r="A54" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="B54" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C54" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D54" t="s">
         <v>3</v>
@@ -6075,7 +6219,7 @@
         <v>0.000</v>
       </c>
       <c r="S54" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="T54" s="5"/>
       <c r="U54" s="5"/>
@@ -6121,13 +6265,13 @@
     </row>
     <row r="55" spans="1:34">
       <c r="A55" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="B55" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C55" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D55" t="s">
         <v>3</v>
@@ -6175,7 +6319,7 @@
         <v>0.000</v>
       </c>
       <c r="S55" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
       <c r="T55" s="5"/>
       <c r="U55" s="5"/>
@@ -6221,13 +6365,13 @@
     </row>
     <row r="56" spans="1:34">
       <c r="A56" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
       <c r="B56" t="s">
         <v>17</v>
       </c>
       <c r="C56" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="D56" t="s">
         <v>3</v>
@@ -6275,7 +6419,7 @@
         <v>0.000</v>
       </c>
       <c r="S56" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="T56" s="5"/>
       <c r="U56" s="5"/>
@@ -6321,13 +6465,13 @@
     </row>
     <row r="57" spans="1:34">
       <c r="A57" t="s">
-        <v>131</v>
+        <v>166</v>
       </c>
       <c r="B57" t="s">
-        <v>17</v>
+        <v>127</v>
       </c>
       <c r="C57" t="s">
-        <v>58</v>
+        <v>128</v>
       </c>
       <c r="D57" t="s">
         <v>3</v>
@@ -6375,7 +6519,7 @@
         <v>0.000</v>
       </c>
       <c r="S57" t="s">
-        <v>132</v>
+        <v>167</v>
       </c>
       <c r="T57" s="5"/>
       <c r="U57" s="5"/>
@@ -6421,13 +6565,13 @@
     </row>
     <row r="58" spans="1:34">
       <c r="A58" t="s">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="B58" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C58" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D58" t="s">
         <v>3</v>
@@ -6475,7 +6619,7 @@
         <v>0.000</v>
       </c>
       <c r="S58" t="s">
-        <v>134</v>
+        <v>169</v>
       </c>
       <c r="T58" s="5"/>
       <c r="U58" s="5"/>
@@ -6521,13 +6665,13 @@
     </row>
     <row r="59" spans="1:34">
       <c r="A59" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="B59" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C59" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D59" t="s">
         <v>3</v>
@@ -6575,7 +6719,7 @@
         <v>0.000</v>
       </c>
       <c r="S59" t="s">
-        <v>136</v>
+        <v>171</v>
       </c>
       <c r="T59" s="5"/>
       <c r="U59" s="5"/>
@@ -6621,13 +6765,13 @@
     </row>
     <row r="60" spans="1:34">
       <c r="A60" t="s">
-        <v>137</v>
+        <v>172</v>
       </c>
       <c r="B60" t="s">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="C60" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
         <v>3</v>
@@ -6675,7 +6819,7 @@
         <v>0.000</v>
       </c>
       <c r="S60" t="s">
-        <v>138</v>
+        <v>173</v>
       </c>
       <c r="T60" s="5"/>
       <c r="U60" s="5"/>
@@ -6721,13 +6865,13 @@
     </row>
     <row r="61" spans="1:34">
       <c r="A61" t="s">
-        <v>139</v>
+        <v>174</v>
       </c>
       <c r="B61" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="C61" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D61" t="s">
         <v>3</v>
@@ -6736,10 +6880,10 @@
         <v>4</v>
       </c>
       <c r="F61" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="G61" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H61" s="2">
         <v>1</v>
@@ -6748,13 +6892,13 @@
         <v>7</v>
       </c>
       <c r="J61" s="3">
-        <v>1.0</v>
+        <v>1.5</v>
       </c>
       <c r="K61" s="3">
-        <v>1.0</v>
+        <v>1.5</v>
       </c>
       <c r="L61" s="3">
-        <v>1.0</v>
+        <v>1.5</v>
       </c>
       <c r="M61" t="s">
         <v>8</v>
@@ -6775,7 +6919,7 @@
         <v>0.000</v>
       </c>
       <c r="S61" t="s">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="T61" s="5"/>
       <c r="U61" s="5"/>
@@ -6821,13 +6965,13 @@
     </row>
     <row r="62" spans="1:34">
       <c r="A62" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="B62" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="C62" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="D62" t="s">
         <v>3</v>
@@ -6836,10 +6980,10 @@
         <v>4</v>
       </c>
       <c r="F62" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G62" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H62" s="2">
         <v>1</v>
@@ -6848,13 +6992,13 @@
         <v>7</v>
       </c>
       <c r="J62" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="K62" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="L62" s="3">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="M62" t="s">
         <v>8</v>
@@ -6875,7 +7019,7 @@
         <v>0.000</v>
       </c>
       <c r="S62" t="s">
-        <v>141</v>
+        <v>177</v>
       </c>
       <c r="T62" s="5"/>
       <c r="U62" s="5"/>
@@ -6921,13 +7065,13 @@
     </row>
     <row r="63" spans="1:34">
       <c r="A63" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="B63" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="C63" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="D63" t="s">
         <v>3</v>
@@ -6936,10 +7080,10 @@
         <v>4</v>
       </c>
       <c r="F63" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G63" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="H63" s="2">
         <v>1</v>
@@ -6948,13 +7092,13 @@
         <v>7</v>
       </c>
       <c r="J63" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K63" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L63" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M63" t="s">
         <v>8</v>
@@ -6975,7 +7119,7 @@
         <v>0.000</v>
       </c>
       <c r="S63" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
       <c r="T63" s="5"/>
       <c r="U63" s="5"/>
@@ -7021,13 +7165,13 @@
     </row>
     <row r="64" spans="1:34">
       <c r="A64" t="s">
-        <v>139</v>
+        <v>180</v>
       </c>
       <c r="B64" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="C64" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="D64" t="s">
         <v>3</v>
@@ -7036,10 +7180,10 @@
         <v>4</v>
       </c>
       <c r="F64" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="G64" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H64" s="2">
         <v>1</v>
@@ -7048,13 +7192,13 @@
         <v>7</v>
       </c>
       <c r="J64" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="K64" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="L64" s="3">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="M64" t="s">
         <v>8</v>
@@ -7075,7 +7219,7 @@
         <v>0.000</v>
       </c>
       <c r="S64" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="T64" s="5"/>
       <c r="U64" s="5"/>
@@ -7121,13 +7265,13 @@
     </row>
     <row r="65" spans="1:34">
       <c r="A65" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C65" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D65" t="s">
         <v>3</v>
@@ -7175,7 +7319,7 @@
         <v>0.000</v>
       </c>
       <c r="S65" t="s">
-        <v>145</v>
+        <v>183</v>
       </c>
       <c r="T65" s="5"/>
       <c r="U65" s="5"/>
@@ -7221,13 +7365,13 @@
     </row>
     <row r="66" spans="1:34">
       <c r="A66" t="s">
-        <v>146</v>
+        <v>184</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C66" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D66" t="s">
         <v>3</v>
@@ -7275,7 +7419,7 @@
         <v>0.000</v>
       </c>
       <c r="S66" t="s">
-        <v>147</v>
+        <v>185</v>
       </c>
       <c r="T66" s="5"/>
       <c r="U66" s="5"/>
@@ -7321,13 +7465,13 @@
     </row>
     <row r="67" spans="1:34">
       <c r="A67" t="s">
-        <v>148</v>
+        <v>186</v>
       </c>
       <c r="B67" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C67" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D67" t="s">
         <v>3</v>
@@ -7375,7 +7519,7 @@
         <v>0.000</v>
       </c>
       <c r="S67" t="s">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="T67" s="5"/>
       <c r="U67" s="5"/>
@@ -7416,6 +7560,506 @@
         <v>3</v>
       </c>
       <c r="AH67" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:34">
+      <c r="A68" t="s">
+        <v>188</v>
+      </c>
+      <c r="B68" t="s">
+        <v>134</v>
+      </c>
+      <c r="C68" t="s">
+        <v>79</v>
+      </c>
+      <c r="D68" t="s">
+        <v>3</v>
+      </c>
+      <c r="E68" t="s">
+        <v>4</v>
+      </c>
+      <c r="F68" t="s">
+        <v>19</v>
+      </c>
+      <c r="G68" t="s">
+        <v>20</v>
+      </c>
+      <c r="H68" s="2">
+        <v>1</v>
+      </c>
+      <c r="I68" t="s">
+        <v>7</v>
+      </c>
+      <c r="J68" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="K68" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="L68" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M68" t="s">
+        <v>8</v>
+      </c>
+      <c r="N68" s="2">
+        <v>0</v>
+      </c>
+      <c r="O68" s="2">
+        <v>0</v>
+      </c>
+      <c r="P68" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="Q68" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="R68" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="S68" t="s">
+        <v>189</v>
+      </c>
+      <c r="T68" s="5"/>
+      <c r="U68" s="5"/>
+      <c r="V68" t="s">
+        <v>10</v>
+      </c>
+      <c r="W68" t="s">
+        <v>3</v>
+      </c>
+      <c r="X68" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y68" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG68" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH68" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:34">
+      <c r="A69" t="s">
+        <v>190</v>
+      </c>
+      <c r="B69" t="s">
+        <v>134</v>
+      </c>
+      <c r="C69" t="s">
+        <v>79</v>
+      </c>
+      <c r="D69" t="s">
+        <v>3</v>
+      </c>
+      <c r="E69" t="s">
+        <v>4</v>
+      </c>
+      <c r="F69" t="s">
+        <v>19</v>
+      </c>
+      <c r="G69" t="s">
+        <v>20</v>
+      </c>
+      <c r="H69" s="2">
+        <v>1</v>
+      </c>
+      <c r="I69" t="s">
+        <v>7</v>
+      </c>
+      <c r="J69" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="K69" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="L69" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M69" t="s">
+        <v>8</v>
+      </c>
+      <c r="N69" s="2">
+        <v>0</v>
+      </c>
+      <c r="O69" s="2">
+        <v>0</v>
+      </c>
+      <c r="P69" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="Q69" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="R69" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="S69" t="s">
+        <v>191</v>
+      </c>
+      <c r="T69" s="5"/>
+      <c r="U69" s="5"/>
+      <c r="V69" t="s">
+        <v>10</v>
+      </c>
+      <c r="W69" t="s">
+        <v>3</v>
+      </c>
+      <c r="X69" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y69" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH69" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:34">
+      <c r="A70" t="s">
+        <v>192</v>
+      </c>
+      <c r="B70" t="s">
+        <v>134</v>
+      </c>
+      <c r="C70" t="s">
+        <v>79</v>
+      </c>
+      <c r="D70" t="s">
+        <v>3</v>
+      </c>
+      <c r="E70" t="s">
+        <v>4</v>
+      </c>
+      <c r="F70" t="s">
+        <v>19</v>
+      </c>
+      <c r="G70" t="s">
+        <v>20</v>
+      </c>
+      <c r="H70" s="2">
+        <v>1</v>
+      </c>
+      <c r="I70" t="s">
+        <v>7</v>
+      </c>
+      <c r="J70" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="K70" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="L70" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M70" t="s">
+        <v>8</v>
+      </c>
+      <c r="N70" s="2">
+        <v>0</v>
+      </c>
+      <c r="O70" s="2">
+        <v>0</v>
+      </c>
+      <c r="P70" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="Q70" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="R70" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="S70" t="s">
+        <v>193</v>
+      </c>
+      <c r="T70" s="5"/>
+      <c r="U70" s="5"/>
+      <c r="V70" t="s">
+        <v>10</v>
+      </c>
+      <c r="W70" t="s">
+        <v>3</v>
+      </c>
+      <c r="X70" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y70" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG70" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH70" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:34">
+      <c r="A71" t="s">
+        <v>194</v>
+      </c>
+      <c r="B71" t="s">
+        <v>134</v>
+      </c>
+      <c r="C71" t="s">
+        <v>79</v>
+      </c>
+      <c r="D71" t="s">
+        <v>3</v>
+      </c>
+      <c r="E71" t="s">
+        <v>4</v>
+      </c>
+      <c r="F71" t="s">
+        <v>19</v>
+      </c>
+      <c r="G71" t="s">
+        <v>20</v>
+      </c>
+      <c r="H71" s="2">
+        <v>1</v>
+      </c>
+      <c r="I71" t="s">
+        <v>7</v>
+      </c>
+      <c r="J71" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="K71" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="L71" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M71" t="s">
+        <v>8</v>
+      </c>
+      <c r="N71" s="2">
+        <v>0</v>
+      </c>
+      <c r="O71" s="2">
+        <v>0</v>
+      </c>
+      <c r="P71" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="Q71" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="R71" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="S71" t="s">
+        <v>195</v>
+      </c>
+      <c r="T71" s="5"/>
+      <c r="U71" s="5"/>
+      <c r="V71" t="s">
+        <v>10</v>
+      </c>
+      <c r="W71" t="s">
+        <v>3</v>
+      </c>
+      <c r="X71" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y71" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG71" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH71" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:34">
+      <c r="A72" t="s">
+        <v>196</v>
+      </c>
+      <c r="B72" t="s">
+        <v>134</v>
+      </c>
+      <c r="C72" t="s">
+        <v>79</v>
+      </c>
+      <c r="D72" t="s">
+        <v>3</v>
+      </c>
+      <c r="E72" t="s">
+        <v>4</v>
+      </c>
+      <c r="F72" t="s">
+        <v>19</v>
+      </c>
+      <c r="G72" t="s">
+        <v>20</v>
+      </c>
+      <c r="H72" s="2">
+        <v>1</v>
+      </c>
+      <c r="I72" t="s">
+        <v>7</v>
+      </c>
+      <c r="J72" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="K72" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="L72" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M72" t="s">
+        <v>8</v>
+      </c>
+      <c r="N72" s="2">
+        <v>0</v>
+      </c>
+      <c r="O72" s="2">
+        <v>0</v>
+      </c>
+      <c r="P72" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="Q72" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="R72" s="4">
+        <v>0.000</v>
+      </c>
+      <c r="S72" t="s">
+        <v>197</v>
+      </c>
+      <c r="T72" s="5"/>
+      <c r="U72" s="5"/>
+      <c r="V72" t="s">
+        <v>10</v>
+      </c>
+      <c r="W72" t="s">
+        <v>3</v>
+      </c>
+      <c r="X72" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y72" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG72" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH72" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>